<commit_message>
fix(afb): adjust text in statistics template
</commit_message>
<xml_diff>
--- a/django/camac/statistics/config/kt_ag/work-items_service-afb.xlsx
+++ b/django/camac/statistics/config/kt_ag/work-items_service-afb.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9672EC8-0B5B-4193-B0ED-6A25DE1E7EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CD1F0F9-A9CB-4405-B522-A1E5C78F11FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="33105" windowHeight="17610" tabRatio="816" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1515" windowWidth="28800" windowHeight="14925" tabRatio="816" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="15" r:id="rId8"/>
+    <pivotCache cacheId="7" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -119,9 +119,6 @@
     <t>Zuständige Person</t>
   </si>
   <si>
-    <t>Anzahl fristgerecht erledigte Aufgaben AfB</t>
-  </si>
-  <si>
     <t>Rolle</t>
   </si>
   <si>
@@ -144,6 +141,9 @@
   </si>
   <si>
     <t>Fristgerecht: 0 = nicht fristgerecht, 1 = fristgerecht</t>
+  </si>
+  <si>
+    <t>Anzahl fristgerecht erledigte Aufgaben</t>
   </si>
 </sst>
 </file>
@@ -220,8 +220,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -247,7 +247,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46146.645671296297" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="19" xr:uid="{A57ED19D-C755-44C2-B72B-40B118E6169D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Stoppe Tilo  Extern" refreshedDate="46210.495823032405" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="19" xr:uid="{A57ED19D-C755-44C2-B72B-40B118E6169D}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:O1048576" sheet="Data"/>
   </cacheSource>
@@ -643,7 +643,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AD818D30-AE36-4ACB-A861-394F5C307186}" name="PivotTable3" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AD818D30-AE36-4ACB-A861-394F5C307186}" name="PivotTable3" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:A6" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="15">
     <pivotField dataField="1" showAll="0"/>
@@ -684,7 +684,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{47A99F71-D715-4130-9576-1DA447D613A1}" name="PivotTable4" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{47A99F71-D715-4130-9576-1DA447D613A1}" name="PivotTable4" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A5:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField showAll="0"/>
@@ -749,7 +749,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{152CAD33-7C43-4DE9-8D77-65A9809A8351}" name="PivotTable5" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Fristgerecht-Filter">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{152CAD33-7C43-4DE9-8D77-65A9809A8351}" name="PivotTable5" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Fristgerecht-Filter">
   <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField dataField="1" showAll="0"/>
@@ -816,7 +816,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C25041AB-465F-4D59-A0D5-A4DCE7C22BCC}" name="PivotTable1" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist-und Aufgabenfilter">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C25041AB-465F-4D59-A0D5-A4DCE7C22BCC}" name="PivotTable1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist-und Aufgabenfilter">
   <location ref="A5:B9" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
@@ -884,7 +884,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4600EC44-62F3-4435-955C-85186BE745A1}" name="PivotTable2" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist-und Aufgabenfilter">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4600EC44-62F3-4435-955C-85186BE745A1}" name="PivotTable2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Zuständige Person" colHeaderCaption="Frist-und Aufgabenfilter">
   <location ref="J5:K9" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField dataField="1" showAll="0" defaultSubtotal="0"/>
@@ -952,7 +952,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB42A912-6B73-470A-8FF3-10598728C1BF}" name="PivotTable4" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Rolle" colHeaderCaption="Fristgerecht-Filter">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FB42A912-6B73-470A-8FF3-10598728C1BF}" name="PivotTable4" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Rolle" colHeaderCaption="Fristgerecht-Filter">
   <location ref="J5:L8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField dataField="1" showAll="0"/>
@@ -1019,7 +1019,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C35527E3-4E41-4635-ACA8-0C5A7744445B}" name="PivotTable6" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Rolle" colHeaderCaption="Fristgerecht-Filter">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C35527E3-4E41-4635-ACA8-0C5A7744445B}" name="PivotTable6" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Rolle" colHeaderCaption="Fristgerecht-Filter">
   <location ref="A5:C8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField dataField="1" showAll="0"/>
@@ -1086,7 +1086,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{920585A1-89C8-48F8-85AC-53EA3CF3C46A}" name="PivotTable7" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Rolle">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{920585A1-89C8-48F8-85AC-53EA3CF3C46A}" name="PivotTable7" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Rolle">
   <location ref="A5:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
     <pivotField showAll="0"/>
@@ -1647,11 +1647,11 @@
   <sheetData>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
+      <c r="A6" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1669,7 +1669,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1717,8 +1717,8 @@
       <c r="A1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="9" t="s">
-        <v>33</v>
+      <c r="H1" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -1744,15 +1744,15 @@
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1779,24 +1779,24 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>33</v>
+        <v>26</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>19</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1825,7 +1825,7 @@
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="8"/>
+      <c r="B8" s="9"/>
       <c r="J8" s="2" t="s">
         <v>15</v>
       </c>
@@ -1837,7 +1837,7 @@
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="8"/>
+      <c r="B9" s="9"/>
       <c r="J9" s="2" t="s">
         <v>17</v>
       </c>
@@ -1874,10 +1874,10 @@
   <sheetData>
     <row r="1" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" s="9" t="s">
         <v>33</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1896,7 +1896,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
         <v>15</v>
@@ -1905,7 +1905,7 @@
         <v>17</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K6" t="s">
         <v>15</v>
@@ -1918,8 +1918,8 @@
       <c r="A7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
       <c r="J7" s="2" t="s">
         <v>15</v>
       </c>
@@ -1934,8 +1934,8 @@
       <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
       <c r="J8" s="2" t="s">
         <v>17</v>
       </c>
@@ -1962,12 +1962,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
@@ -1991,26 +1991,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5e238f3b-cf1c-4dc8-b1c3-14677632393c">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="fb274a4b-4ecf-4ae2-a446-66548455045d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100D7FFFCF5F95BC94D9B7DF34B9D0CF76C" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="a8184ac6384f947bbc55bc4d9e1749d1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5e238f3b-cf1c-4dc8-b1c3-14677632393c" xmlns:ns3="a7360a35-2516-4210-888a-7cc8dd0a384d" xmlns:ns4="fb274a4b-4ecf-4ae2-a446-66548455045d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6dc33f40212c2dffa236803017f7661f" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="5e238f3b-cf1c-4dc8-b1c3-14677632393c"/>
@@ -2250,26 +2230,27 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5e238f3b-cf1c-4dc8-b1c3-14677632393c">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="fb274a4b-4ecf-4ae2-a446-66548455045d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10038610-FC0E-4438-92ED-50D46C596A94}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5e238f3b-cf1c-4dc8-b1c3-14677632393c"/>
-    <ds:schemaRef ds:uri="fb274a4b-4ecf-4ae2-a446-66548455045d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C25DC3E-57ED-4CB1-BB3F-A437A2199860}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3181E807-AA15-40C5-8B70-A01DB7520019}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2287,4 +2268,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10038610-FC0E-4438-92ED-50D46C596A94}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5e238f3b-cf1c-4dc8-b1c3-14677632393c"/>
+    <ds:schemaRef ds:uri="fb274a4b-4ecf-4ae2-a446-66548455045d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C25DC3E-57ED-4CB1-BB3F-A437A2199860}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>